<commit_message>
atualização antes de ser feita a troca de PC
</commit_message>
<xml_diff>
--- a/02-Referencias/FOPA/premio_total_por_colaborador_MAI2026.xlsx
+++ b/02-Referencias/FOPA/premio_total_por_colaborador_MAI2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julio.santana\Documents\Projects\Cofre_Trabalho\02-Referencias\FOPA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7285B40-3A8C-4400-ADF1-8ECDBF307F25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8B3EE64-6B90-4FD3-AEE1-04144EE45E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="5" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="200" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -1049,24 +1049,12 @@
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="2">
     <dxf>
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2212,7 +2200,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EB923BD4-24FB-4B16-A8F0-5211B8C4F38D}" name="Tabela dinâmica5" cacheId="200" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EB923BD4-24FB-4B16-A8F0-5211B8C4F38D}" name="Tabela dinâmica5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B66" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField showAll="0"/>
@@ -2488,10 +2476,10 @@
     <dataField name="Soma de premio_total" fld="2" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="4">
+    <format dxfId="1">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="0">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -3384,7 +3372,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
@@ -3436,7 +3424,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>28</v>
       </c>
@@ -3540,7 +3528,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>42</v>
       </c>
@@ -3748,7 +3736,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>75</v>
       </c>
@@ -3826,7 +3814,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>88</v>
       </c>
@@ -3852,7 +3840,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>94</v>
       </c>
@@ -3904,7 +3892,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>99</v>
       </c>
@@ -4008,7 +3996,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>108</v>
       </c>
@@ -4034,7 +4022,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>109</v>
       </c>
@@ -4138,7 +4126,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>118</v>
       </c>
@@ -4190,7 +4178,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>122</v>
       </c>
@@ -4216,7 +4204,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>123</v>
       </c>
@@ -4398,7 +4386,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>140</v>
       </c>
@@ -4450,7 +4438,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>148</v>
       </c>
@@ -4554,7 +4542,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>160</v>
       </c>
@@ -4606,7 +4594,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>163</v>
       </c>
@@ -4632,7 +4620,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
         <v>164</v>
       </c>
@@ -4658,7 +4646,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>165</v>
       </c>
@@ -4684,7 +4672,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
         <v>166</v>
       </c>
@@ -4814,7 +4802,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>173</v>
       </c>
@@ -5022,7 +5010,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>188</v>
       </c>
@@ -5048,7 +5036,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>189</v>
       </c>
@@ -5204,7 +5192,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
         <v>200</v>
       </c>
@@ -5334,7 +5322,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
         <v>207</v>
       </c>
@@ -5360,7 +5348,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="4" t="s">
         <v>208</v>
       </c>
@@ -5386,7 +5374,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
         <v>209</v>
       </c>
@@ -5412,7 +5400,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>210</v>
       </c>
@@ -5490,7 +5478,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>217</v>
       </c>
@@ -5516,7 +5504,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>218</v>
       </c>
@@ -5542,7 +5530,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>220</v>
       </c>
@@ -5594,7 +5582,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>224</v>
       </c>
@@ -5698,7 +5686,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
         <v>228</v>
       </c>
@@ -5724,7 +5712,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>229</v>
       </c>
@@ -6038,9 +6026,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H104" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="7">
+    <filterColumn colId="3">
       <filters>
-        <filter val="BOLETO G&amp;S BARUERI FIL 05 SEGURO DE VIDA COMP JUN26.PDF"/>
+        <filter val="172"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>